<commit_message>
Update soccer trades 2026-08-08 16:03:49 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,110 +531,526 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>9.59075</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.1975</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1786204683</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>48.560759</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-08 17:02:49 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,59 +531,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,23 +651,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -667,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -747,23 +763,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -771,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -816,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -854,12 +878,12 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -875,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -920,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,110 +971,422 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-08 19:02:30 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Vicenza -1.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +650,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio 0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,28 +859,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -914,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -979,23 +971,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1003,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,31 +1075,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,36 +1187,44 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>Vicenza vs Catania</t>
@@ -1226,7 +1242,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,110 +1299,750 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.42844</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786206465</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1.422207</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4.91</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786206249</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>16.298755</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>9.59075</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.1975</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786204683</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>48.560759</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-08 20:02:23 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -675,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,29 +754,29 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio 0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
@@ -802,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,31 +851,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -906,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1003,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Vicenza 0</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1115,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,12 +1187,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1202,22 +1202,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,12 +1299,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1314,12 +1314,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1339,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1384,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,12 +1411,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1426,22 +1426,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1451,27 +1451,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,23 +1523,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,31 +1627,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1659,27 +1667,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1712,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,31 +1739,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1778,7 +1794,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1808,7 +1824,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1834,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,28 +1851,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1867,27 +1883,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1912,17 +1928,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,110 +1955,1086 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.455</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786211540</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>21.978022</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>49.90995</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.7388</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786211170</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>67.56</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>5.48</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786206603</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>18.190871</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.42844</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786206465</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>1.422207</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>4.91</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786206249</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>16.298755</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>9.59075</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.1975</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1786204683</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>48.560759</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 09:02:15 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Arezzo 0</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -667,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -754,22 +770,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -779,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -859,31 +875,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -906,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -971,31 +979,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1115,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1202,22 +1202,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1227,27 +1227,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,17 +1272,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1314,22 +1314,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1426,22 +1426,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Vicenza 0</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1451,27 +1451,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,23 +1523,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1547,7 +1551,11 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1555,27 +1563,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1600,17 +1608,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,12 +1635,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,22 +1650,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1667,27 +1675,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1712,17 +1720,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,12 +1747,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1754,22 +1762,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1794,7 +1802,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1832,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1842,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,28 +1859,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1898,7 +1906,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1928,7 +1936,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1938,7 +1946,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,12 +1963,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1970,22 +1978,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2010,7 +2018,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2040,7 +2048,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2050,7 +2058,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,12 +2075,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2082,22 +2090,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Ascoli Picchio 0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2122,7 +2130,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2152,7 +2160,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2162,7 +2170,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2179,7 +2187,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2187,31 +2195,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Vicenza -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2219,27 +2219,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2264,17 +2264,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2291,7 +2291,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2306,22 +2306,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2403,12 +2403,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2418,22 +2418,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2443,27 +2443,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2488,17 +2488,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2515,31 +2515,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2547,27 +2555,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2592,17 +2600,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2619,7 +2627,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2627,23 +2635,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2651,27 +2667,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2696,17 +2712,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2723,7 +2739,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2731,23 +2747,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2755,27 +2779,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2800,17 +2824,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2851,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2838,12 +2862,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2859,27 +2883,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2904,17 +2928,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,110 +2955,422 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="S27" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 15:03:46 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -698,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +754,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +851,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,31 +963,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1003,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1083,31 +1083,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1130,7 +1122,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,31 +1187,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1242,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1272,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1314,12 +1298,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1384,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1394,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1426,22 +1410,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1451,27 +1435,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1480,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1538,22 +1522,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1563,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1608,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1650,22 +1634,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Vicenza 0</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1675,27 +1659,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1720,17 +1704,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1747,7 +1731,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1762,22 +1746,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1787,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1832,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1859,31 +1843,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1906,7 +1898,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1936,7 +1928,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1946,7 +1938,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,12 +1955,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1978,22 +1970,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2003,27 +1995,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2048,17 +2040,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2075,7 +2067,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2083,19 +2075,15 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2103,11 +2091,7 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio 0</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2160,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2170,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2187,31 +2171,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2219,27 +2211,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2264,17 +2256,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2291,12 +2283,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2306,22 +2298,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Ascoli Picchio 0</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2331,27 +2323,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2376,17 +2368,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2403,39 +2395,31 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2458,7 +2442,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2488,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2498,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2515,7 +2499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2530,22 +2514,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2570,7 +2554,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2600,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2610,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2627,12 +2611,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2642,22 +2626,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2667,27 +2651,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2712,17 +2696,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2739,7 +2723,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2754,7 +2738,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2824,7 +2808,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2834,7 +2818,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2851,31 +2835,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2883,27 +2875,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2928,17 +2920,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2955,7 +2947,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2963,23 +2955,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2987,27 +2987,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3032,17 +3032,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3059,28 +3059,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,28 +3163,28 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>11.94608</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.8538</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -3195,27 +3195,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3240,17 +3240,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204434</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>13.99248</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3267,110 +3267,318 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 18:02:15 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +635,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -667,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,67 +739,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +843,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -866,22 +858,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -906,7 +898,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,12 +955,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -978,22 +970,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1003,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1040,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,59 +1067,67 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,59 +1179,67 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Arezzo -1.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1256,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,12 +1291,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1298,12 +1306,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1313,7 +1321,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1323,27 +1331,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1376,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,12 +1403,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1410,22 +1418,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1435,27 +1443,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,17 +1488,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,12 +1515,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1522,12 +1530,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1537,7 +1545,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1547,27 +1555,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1600,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1627,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,52 +1642,52 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Vicenza 0</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1712,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,52 +1754,52 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1824,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,12 +1851,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1858,22 +1866,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1883,27 +1891,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1928,17 +1936,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,39 +1963,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1995,27 +1995,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,17 +2040,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,28 +2067,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2099,27 +2099,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,12 +2171,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2186,22 +2186,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2211,27 +2211,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2256,17 +2256,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,12 +2283,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2298,52 +2298,52 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio 0</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2368,17 +2368,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2403,23 +2403,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2427,27 +2435,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2472,17 +2480,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,39 +2507,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2539,27 +2539,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2584,17 +2584,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2611,39 +2611,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2666,7 +2658,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2696,7 +2688,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2706,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2723,12 +2715,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2738,22 +2730,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2763,27 +2755,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2808,17 +2800,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2835,12 +2827,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2850,22 +2842,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2875,27 +2867,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2920,17 +2912,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2947,12 +2939,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2962,22 +2954,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2987,27 +2979,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3032,17 +3024,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3059,23 +3051,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3083,7 +3079,11 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Vicenza 0</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3091,27 +3091,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3136,17 +3136,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,31 +3163,39 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3195,27 +3203,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3240,17 +3248,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3267,31 +3275,39 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1.5</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3314,7 +3330,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3344,7 +3360,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3354,7 +3370,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3371,59 +3387,67 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3448,17 +3472,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,110 +3499,1518 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>27.61</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.2363</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786215506</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>116.867725</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>436.64999</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.5663</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1786214910</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>771.12581</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>13.08</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.5413</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1786214365</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>24.166282</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>3.28999</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.7175</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1786214242</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>4.585352</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.455</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1786211540</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>21.978022</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>49.90995</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.7388</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1786211170</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>67.56</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>5.48</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1786206603</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>18.190871</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0.42844</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1786206465</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>1.422207</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>4.91</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1786206249</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>16.298755</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>9.59075</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.1975</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1786204683</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>48.560759</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="S42" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 19:02:40 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -578,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -646,17 +654,17 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,28 +747,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -786,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,27 +851,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -871,11 +875,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -883,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,12 +955,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -970,22 +970,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -995,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1040,17 +1040,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,12 +1179,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1194,12 +1194,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1219,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1306,22 +1306,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1418,22 +1418,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,7 +1515,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1530,22 +1530,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,7 +1627,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1642,22 +1642,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1667,27 +1667,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1712,17 +1712,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1754,22 +1754,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1891,27 +1891,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1936,17 +1936,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,23 +1963,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1987,7 +1991,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Union Brescia</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2040,7 +2048,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2050,7 +2058,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,7 +2075,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2144,7 +2152,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2171,44 +2179,36 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>Arezzo vs Union Brescia</t>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,12 +2283,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2298,22 +2298,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2507,59 +2507,67 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2584,17 +2592,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2611,7 +2619,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2622,7 +2630,7 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2658,7 +2666,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2698,7 +2706,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2723,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2723,31 +2731,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2842,12 +2842,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3051,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3066,52 +3066,52 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Vicenza 0</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3136,17 +3136,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3163,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3193,24 +3193,24 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>Vicenza 0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>Vicenza</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Vicenza vs Catania</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Catania</t>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,22 +3290,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3315,27 +3315,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3360,17 +3360,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,22 +3402,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,36 +3499,44 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
@@ -3546,7 +3554,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3576,7 +3584,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3586,7 +3594,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3603,7 +3611,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3611,31 +3619,23 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3643,27 +3643,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3688,17 +3688,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3715,7 +3715,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3730,52 +3730,52 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio 0</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3800,17 +3800,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3827,31 +3827,39 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3874,7 +3882,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3904,7 +3912,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3914,7 +3922,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3931,7 +3939,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3939,31 +3947,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3971,27 +3971,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4016,17 +4016,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4043,12 +4043,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4058,22 +4058,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4083,27 +4083,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4128,17 +4128,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4155,12 +4155,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4170,22 +4170,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4195,27 +4195,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4240,17 +4240,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4267,7 +4267,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4379,7 +4379,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4491,59 +4491,67 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4568,17 +4576,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4595,28 +4603,28 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -4642,7 +4650,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4672,7 +4680,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4682,7 +4690,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4699,7 +4707,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4710,7 +4718,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>11.94608</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4776,7 +4784,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786204434</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4786,7 +4794,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>13.99248</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4803,28 +4811,28 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>46.42999</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.8538</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -4835,27 +4843,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4880,17 +4888,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204373</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>54.38359</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4907,110 +4915,214 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 20:03:12 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
+          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.29</t>
+          <t>34.28</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4563</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786301791</t>
+          <t>1786303449</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>22.553425</t>
+          <t>62.327273</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,28 +635,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>22.73178</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -690,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786302954</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>313.541793</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,23 +739,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>14.33585</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -779,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786302861</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>197.735862</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +843,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -859,23 +851,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -883,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -963,19 +963,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -983,34 +979,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Arezzo vs Union Brescia</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Arezzo</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Union Brescia</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Arezzo vs Union Brescia</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Arezzo</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1040,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,39 +1059,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Benevento Calcio -1.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1122,7 +1106,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1136,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1146,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,39 +1163,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Benevento Calcio -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1234,7 +1210,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1240,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1250,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1267,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1306,22 +1282,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1346,7 +1322,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1376,7 +1352,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1362,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,12 +1379,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1418,22 +1394,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1443,27 +1419,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1488,17 +1464,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,12 +1491,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1530,12 +1506,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1545,7 +1521,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1555,27 +1531,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1600,17 +1576,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,7 +1603,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1642,22 +1618,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1682,7 +1658,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1688,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1698,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,7 +1715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1754,22 +1730,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1779,27 +1755,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1824,17 +1800,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1827,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1866,22 +1842,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1891,27 +1867,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1936,17 +1912,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,7 +1939,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1978,47 +1954,47 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Arezzo vs Union Brescia</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Arezzo</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t>Union Brescia</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Arezzo vs Union Brescia</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Arezzo</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2048,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2058,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2075,31 +2051,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1.5</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2107,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2152,17 +2136,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2179,23 +2163,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2203,7 +2191,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2211,27 +2203,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2256,17 +2248,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2298,22 +2290,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Arezzo 0</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2338,7 +2330,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2368,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,39 +2387,31 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2450,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2480,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2490,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2507,39 +2491,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2562,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2592,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2602,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2619,23 +2595,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2643,7 +2623,11 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Arezzo 0</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2651,27 +2635,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2696,17 +2680,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2723,31 +2707,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2755,27 +2747,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2800,17 +2792,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,12 +2819,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2842,22 +2834,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2867,27 +2859,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2912,17 +2904,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2939,7 +2931,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2947,31 +2939,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2994,7 +2978,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3024,7 +3008,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3034,7 +3018,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3051,7 +3035,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3059,31 +3043,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3106,7 +3082,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3136,7 +3112,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3146,7 +3122,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3163,7 +3139,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3178,22 +3154,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3203,27 +3179,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3248,17 +3224,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3275,7 +3251,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3290,22 +3266,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3315,27 +3291,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3360,17 +3336,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3387,7 +3363,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3402,22 +3378,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3442,7 +3418,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3472,7 +3448,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3482,7 +3458,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3475,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3514,22 +3490,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Vicenza 0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3539,27 +3515,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3584,17 +3560,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3611,23 +3587,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3635,7 +3615,11 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3643,27 +3627,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3688,17 +3672,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3715,12 +3699,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3730,22 +3714,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3755,27 +3739,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3800,17 +3784,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3827,12 +3811,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3842,22 +3826,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3882,7 +3866,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3912,7 +3896,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3922,7 +3906,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3939,28 +3923,28 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3986,7 +3970,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4016,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4026,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4043,12 +4027,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4058,22 +4042,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4098,7 +4082,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4128,7 +4112,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4138,7 +4122,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4155,12 +4139,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4170,22 +4154,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Ascoli Picchio 0</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4210,7 +4194,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4240,7 +4224,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4250,7 +4234,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4267,7 +4251,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4275,31 +4259,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Vicenza -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4307,27 +4283,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4352,17 +4328,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4379,7 +4355,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4394,22 +4370,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4434,7 +4410,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4464,7 +4440,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4474,7 +4450,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4491,12 +4467,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4506,22 +4482,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4531,27 +4507,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4576,17 +4552,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4603,31 +4579,39 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4635,27 +4619,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4680,17 +4664,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4707,7 +4691,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4715,23 +4699,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4739,27 +4731,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4784,17 +4776,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4811,7 +4803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4819,23 +4811,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4843,27 +4843,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4888,17 +4888,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4915,7 +4915,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4926,12 +4926,12 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4947,27 +4947,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4992,17 +4992,17 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5019,110 +5019,422 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-09 23:02:39 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
+          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>34.28</t>
+          <t>98.93</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.5725</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
+          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786303449</t>
+          <t>1786308240</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>62.327273</t>
+          <t>172.803493</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +643,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
+          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22.73178</t>
+          <t>34.28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -682,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
+          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786302954</t>
+          <t>1786303449</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>313.541793</t>
+          <t>62.327273</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
+          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,7 +758,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.33585</t>
+          <t>22.73178</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786302861</t>
+          <t>1786302954</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>197.735862</t>
+          <t>313.541793</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,39 +851,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
+          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.29</t>
+          <t>14.33585</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4563</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -898,7 +898,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786301791</t>
+          <t>1786302861</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>22.553425</t>
+          <t>197.735862</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,31 +955,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1002,7 +1010,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1032,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,7 +1067,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1070,17 +1078,17 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1091,27 +1099,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1136,17 +1144,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,28 +1171,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1210,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1240,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1250,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1267,27 +1275,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1295,11 +1299,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1307,27 +1307,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1352,17 +1352,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,12 +1379,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1394,22 +1394,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1419,27 +1419,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1464,17 +1464,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,12 +1491,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,12 +1603,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1643,27 +1643,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1688,17 +1688,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,7 +1715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1730,22 +1730,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,7 +1827,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1842,22 +1842,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,7 +1939,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1954,22 +1954,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,7 +2051,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2066,22 +2066,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2091,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2136,17 +2136,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,7 +2163,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2178,22 +2178,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,7 +2275,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2290,12 +2290,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2315,27 +2315,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,17 +2360,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,23 +2387,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2411,7 +2415,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Union Brescia</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2464,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2568,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2595,39 +2603,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,12 +2707,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2722,22 +2722,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2819,7 +2819,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,31 +2931,39 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2963,27 +2971,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3008,17 +3016,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3035,7 +3043,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3046,7 +3054,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3082,7 +3090,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3122,7 +3130,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3139,7 +3147,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3147,31 +3155,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3266,12 +3266,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3363,7 +3363,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3378,12 +3378,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,7 +3475,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3490,22 +3490,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3515,27 +3515,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3560,17 +3560,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3617,24 +3617,24 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>Vicenza 0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
           <t>Vicenza</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Vicenza vs Catania</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>Catania</t>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,7 +3699,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3714,22 +3714,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3739,27 +3739,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3784,17 +3784,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3811,7 +3811,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3826,22 +3826,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3923,31 +3923,39 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3970,7 +3978,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4000,7 +4008,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4010,7 +4018,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4035,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4035,31 +4043,23 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4067,27 +4067,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4112,17 +4112,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4154,22 +4154,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4179,27 +4179,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4224,17 +4224,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,31 +4251,39 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4298,7 +4306,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4328,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4338,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4355,7 +4363,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4363,31 +4371,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4395,27 +4395,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4440,17 +4440,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4467,12 +4467,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4482,22 +4482,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4507,27 +4507,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4552,17 +4552,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,12 +4579,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4594,22 +4594,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4619,27 +4619,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4664,17 +4664,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4691,7 +4691,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4706,7 +4706,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4803,7 +4803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4915,31 +4915,39 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4947,27 +4955,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4992,17 +5000,17 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5019,28 +5027,28 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -5066,7 +5074,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5096,7 +5104,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5106,7 +5114,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5131,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5134,7 +5142,7 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>11.94608</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5200,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786204434</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5210,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>13.99248</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5227,28 +5235,28 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>46.42999</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.8538</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -5259,27 +5267,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5304,17 +5312,17 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204373</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>54.38359</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5331,110 +5339,214 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S47" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="V47" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-12 19:03:05 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
+          <t>0xd64487136d220bcde0c34443c28dae20b7ce8df92715349e80439bb3add91afd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x960070fC76573ff9c086dB473f99CA99ea914dd6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>98.93</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5725</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Benevento Calcio -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Udinese Calcio vs Padova</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Udinese Calcio</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
+          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19758479</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786308240</t>
+          <t>1786559970</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786811400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>172.803493</t>
+          <t>9.056604</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +635,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
+          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>34.28</t>
+          <t>98.93</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.5725</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
+          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786303449</t>
+          <t>1786308240</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>62.327273</t>
+          <t>172.803493</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,28 +747,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
+          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>22.73178</t>
+          <t>34.28</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -794,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
+          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786302954</t>
+          <t>1786303449</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>313.541793</t>
+          <t>62.327273</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
+          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -862,7 +862,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>14.33585</t>
+          <t>22.73178</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786302861</t>
+          <t>1786302954</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>197.735862</t>
+          <t>313.541793</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,39 +955,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
+          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.29</t>
+          <t>14.33585</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4563</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1010,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1040,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786301791</t>
+          <t>1786302861</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>22.553425</t>
+          <t>197.735862</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,31 +1059,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1182,17 +1182,17 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1203,27 +1203,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1248,17 +1248,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,28 +1275,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,27 +1379,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1407,11 +1403,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1419,27 +1411,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1464,17 +1456,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,12 +1483,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1506,22 +1498,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1531,27 +1523,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1576,17 +1568,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,12 +1595,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1618,7 +1610,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1688,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1698,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1730,12 +1722,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1745,7 +1737,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1755,27 +1747,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1800,17 +1792,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,7 +1819,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1842,22 +1834,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1882,7 +1874,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1922,7 +1914,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,7 +1931,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1954,22 +1946,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1994,7 +1986,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2024,7 +2016,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2026,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,7 +2043,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2066,22 +2058,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2106,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2136,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2146,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,7 +2155,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2178,22 +2170,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2203,27 +2195,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2248,17 +2240,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,7 +2267,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2290,22 +2282,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2330,7 +2322,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2360,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,7 +2379,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2402,12 +2394,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2417,7 +2409,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2427,27 +2419,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2472,17 +2464,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,23 +2491,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2523,7 +2519,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Union Brescia</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2707,39 +2707,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2762,7 +2754,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2792,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2802,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2819,12 +2811,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2834,22 +2826,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2874,7 +2866,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2904,7 +2896,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2906,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,7 +2923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2946,7 +2938,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3016,7 +3008,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3026,7 +3018,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,31 +3035,39 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3075,27 +3075,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3120,17 +3120,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3158,7 +3158,7 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3259,31 +3259,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3306,7 +3298,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3336,7 +3328,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3346,7 +3338,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3363,7 +3355,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3378,12 +3370,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3448,7 +3440,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3458,7 +3450,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,7 +3467,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3490,12 +3482,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3560,7 +3552,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3570,7 +3562,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,7 +3579,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3602,22 +3594,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3627,27 +3619,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3672,17 +3664,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,7 +3691,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3714,7 +3706,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3729,24 +3721,24 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>Vicenza 0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
           <t>Vicenza</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Vicenza vs Catania</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>Catania</t>
@@ -3754,7 +3746,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3794,7 +3786,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3811,7 +3803,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3826,22 +3818,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3851,27 +3843,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3896,17 +3888,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3923,7 +3915,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3938,22 +3930,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3978,7 +3970,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4008,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4018,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4035,31 +4027,39 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4147,31 +4147,23 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4179,27 +4171,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4224,17 +4216,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,7 +4243,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4266,22 +4258,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4291,27 +4283,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4336,17 +4328,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,31 +4355,39 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4410,7 +4410,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4467,7 +4467,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4475,31 +4475,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4507,27 +4499,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4552,17 +4544,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4579,12 +4571,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4594,22 +4586,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4619,27 +4611,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4664,17 +4656,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4691,12 +4683,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4706,22 +4698,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4731,27 +4723,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4776,17 +4768,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4803,7 +4795,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4818,7 +4810,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4888,7 +4880,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4898,7 +4890,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4915,7 +4907,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4930,7 +4922,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -5000,7 +4992,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5010,7 +5002,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5027,31 +5019,39 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5059,27 +5059,27 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -5104,17 +5104,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5131,28 +5131,28 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,7 +5235,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5246,7 +5246,7 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>11.94608</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786204434</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>13.99248</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5339,28 +5339,28 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>46.42999</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.8538</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -5371,27 +5371,27 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -5416,17 +5416,17 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204373</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>54.38359</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5443,110 +5443,214 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-13 12:03:44 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd64487136d220bcde0c34443c28dae20b7ce8df92715349e80439bb3add91afd</t>
+          <t>0x066ffec83e87f611402a754498c12bc6703ec2b4b1838ef49ab5112ae75390ef</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x960070fC76573ff9c086dB473f99CA99ea914dd6</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>67.75</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Udinese Calcio vs Padova</t>
+          <t>Fiorentina vs Benevento Calcio</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Udinese Calcio</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Padova</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
+          <t>0x466e5e0d982ed66aa368c8de6cbe0433d76f7b199a295fb9a3962661d07d8e0c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19758479</t>
+          <t>L19755776</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786559970</t>
+          <t>1786605663</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786811400</t>
+          <t>1786734900</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>9.056604</t>
+          <t>289.839572</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
+          <t>0xd64487136d220bcde0c34443c28dae20b7ce8df92715349e80439bb3add91afd</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x960070fC76573ff9c086dB473f99CA99ea914dd6</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>98.93</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5725</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Benevento Calcio -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -675,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Udinese Calcio vs Padova</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Udinese Calcio</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
+          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19758479</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786308240</t>
+          <t>1786559970</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786811400</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>172.803493</t>
+          <t>9.056604</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,31 +739,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
+          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>34.28</t>
+          <t>98.93</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.5725</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -779,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
+          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786303449</t>
+          <t>1786308240</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>62.327273</t>
+          <t>172.803493</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,28 +851,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
+          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22.73178</t>
+          <t>34.28</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
+          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786302954</t>
+          <t>1786303449</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>313.541793</t>
+          <t>62.327273</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
+          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -966,7 +966,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14.33585</t>
+          <t>22.73178</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786302861</t>
+          <t>1786302954</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>197.735862</t>
+          <t>313.541793</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,39 +1059,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
+          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.29</t>
+          <t>14.33585</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4563</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1114,7 +1106,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1144,7 +1136,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786301791</t>
+          <t>1786302861</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1146,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>22.553425</t>
+          <t>197.735862</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,31 +1163,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,7 +1275,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1286,17 +1286,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1307,27 +1307,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1352,17 +1352,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,28 +1379,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1483,27 +1483,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1511,11 +1507,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1523,27 +1515,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1568,17 +1560,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,12 +1587,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1610,22 +1602,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1635,27 +1627,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1680,17 +1672,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,12 +1699,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1722,7 +1714,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1792,7 +1784,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1794,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,12 +1811,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1834,12 +1826,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1849,7 +1841,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1859,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1904,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,7 +1923,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1946,22 +1938,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1986,7 +1978,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2026,7 +2018,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2043,7 +2035,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2058,22 +2050,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2098,7 +2090,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2147,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2170,22 +2162,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2210,7 +2202,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2240,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,7 +2259,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2282,22 +2274,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2307,27 +2299,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2352,17 +2344,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,7 +2371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2394,22 +2386,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2434,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2464,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2483,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2506,12 +2498,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2521,7 +2513,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2531,27 +2523,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2576,17 +2568,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,23 +2595,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2627,7 +2623,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Union Brescia</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,7 +2707,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2811,39 +2811,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Arezzo 0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2866,7 +2858,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2896,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2906,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2923,12 +2915,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2938,22 +2930,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2978,7 +2970,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3008,7 +3000,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3018,7 +3010,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3035,7 +3027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3050,7 +3042,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3120,7 +3112,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3130,7 +3122,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3147,31 +3139,39 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3179,27 +3179,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3224,17 +3224,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3262,7 +3262,7 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3355,7 +3355,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3363,31 +3363,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Ascoli Picchio -1</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3410,7 +3402,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3440,7 +3432,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3450,7 +3442,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3467,7 +3459,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3482,12 +3474,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3552,7 +3544,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3562,7 +3554,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3579,7 +3571,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3594,12 +3586,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3664,7 +3656,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3674,7 +3666,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3691,7 +3683,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3706,22 +3698,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Vicenza 0</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3731,27 +3723,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3776,17 +3768,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,7 +3795,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3818,7 +3810,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3833,24 +3825,24 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>Vicenza 0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
           <t>Vicenza</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Vicenza vs Catania</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>Catania</t>
@@ -3858,7 +3850,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3898,7 +3890,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,7 +3907,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3930,22 +3922,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3955,27 +3947,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4000,17 +3992,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4019,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4042,22 +4034,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Ascoli Picchio -1.5</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4082,7 +4074,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4112,7 +4104,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4122,7 +4114,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,31 +4131,39 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4243,7 +4243,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4251,31 +4251,23 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4283,27 +4275,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4328,17 +4320,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4355,7 +4347,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4370,22 +4362,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4395,27 +4387,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4440,17 +4432,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4467,31 +4459,39 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio 0</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4571,7 +4571,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4579,31 +4579,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4611,27 +4603,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4656,17 +4648,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4683,12 +4675,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4698,22 +4690,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4723,27 +4715,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4768,17 +4760,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4795,12 +4787,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4810,22 +4802,22 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -4835,27 +4827,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4880,17 +4872,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4907,7 +4899,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4922,7 +4914,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4992,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5002,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5019,7 +5011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5034,7 +5026,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5104,7 +5096,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5114,7 +5106,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5131,31 +5123,39 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5163,27 +5163,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5208,17 +5208,17 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786206249</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>16.298755</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,28 +5235,28 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>9.59075</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.1975</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786204683</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>48.560759</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5339,7 +5339,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5350,7 +5350,7 @@
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>11.94608</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786204434</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>13.99248</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5443,28 +5443,28 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>46.42999</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.8538</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -5475,27 +5475,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5520,17 +5520,17 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786204373</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>54.38359</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5547,110 +5547,214 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S49" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T49" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
+      <c r="V49" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-13 18:04:59 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Coppa Italia/trades.xlsx
+++ b/data/sxbet/ligas/Coppa Italia/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V49"/>
+  <dimension ref="A1:V54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x066ffec83e87f611402a754498c12bc6703ec2b4b1838ef49ab5112ae75390ef</t>
+          <t>0xe2cbbd60f019c5760479a08511801034d5b50a72031d97189fedf1bb3b61b51e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,15 +539,19 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>67.75</t>
+          <t>222.31999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2338</t>
+          <t>1.7037</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Udinese Calcio</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Fiorentina vs Benevento Calcio</t>
+          <t>Udinese Calcio vs Padova</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Udinese Calcio</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x466e5e0d982ed66aa368c8de6cbe0433d76f7b199a295fb9a3962661d07d8e0c</t>
+          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19755776</t>
+          <t>L19758479</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786605663</t>
+          <t>1786642103</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786734900</t>
+          <t>1786811400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>289.839572</t>
+          <t>315.907623</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,28 +643,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xd64487136d220bcde0c34443c28dae20b7ce8df92715349e80439bb3add91afd</t>
+          <t>0xf8aa36c5e4b0c9667086ff19f5381cc07c32ab8da06463cc05b227f4cd6cf473</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x960070fC76573ff9c086dB473f99CA99ea914dd6</t>
+          <t>0x29c4c7668B1f9E7B037b36080Ea8682510C66b0e</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>34.87998</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.7325</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-2)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Udinese Calcio vs Padova</t>
+          <t>Cagliari vs Arezzo</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Udinese Calcio</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Padova</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
+          <t>0x5c005869df336580ac6253f3a8b07c9210ec6611e1b593f446aff688e3881503</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19758479</t>
+          <t>L19763845</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786559970</t>
+          <t>1786641379</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786811400</t>
+          <t>1786725000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>9.056604</t>
+          <t>47.61772</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
+          <t>0x8ec8718ffb04e0ce90d37ffa902e51333a95d8aac782b436ca14bb0f1d1d6b76</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x29c4c7668B1f9E7B037b36080Ea8682510C66b0e</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -754,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>98.93</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5725</t>
+          <t>1.2625</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-2)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1</t>
+          <t>Cagliari -2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -779,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Cagliari vs Arezzo</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
+          <t>0x5c005869df336580ac6253f3a8b07c9210ec6611e1b593f446aff688e3881503</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19763845</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786308240</t>
+          <t>1786641378</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786725000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>172.803493</t>
+          <t>47.619048</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,31 +859,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
+          <t>0xa939fd0abe4695755faa4bb2a7f869126de6c2df9849c52bb96e55dffb4dd9a8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>34.28</t>
+          <t>12.43</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-2)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Cagliari -2</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -883,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Cagliari vs Arezzo</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>Arezzo</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
+          <t>0x5c005869df336580ac6253f3a8b07c9210ec6611e1b593f446aff688e3881503</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19763845</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786303449</t>
+          <t>1786641337</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786725000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>62.327273</t>
+          <t>47.578947</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,28 +971,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
+          <t>0x2f3b2184deba7400673419e62d0eaca5f386d566d051f9e28056a66fdb7783b5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>22.73178</t>
+          <t>12.13</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.4863</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -987,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Cagliari vs Arezzo</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>Arezzo</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
+          <t>0x633539b4e4ddef81c1a23b7f8f66b31324f5f2b22f654f8fb7fe9ddddaf4dbe8</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19763845</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1032,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786302954</t>
+          <t>1786635113</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786725000</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>313.541793</t>
+          <t>24.946015</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,28 +1075,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
+          <t>0x066ffec83e87f611402a754498c12bc6703ec2b4b1838ef49ab5112ae75390ef</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>14.33585</t>
+          <t>67.75</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1091,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Fiorentina vs Benevento Calcio</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
+          <t>0x466e5e0d982ed66aa368c8de6cbe0433d76f7b199a295fb9a3962661d07d8e0c</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19755776</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1136,17 +1152,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786302861</t>
+          <t>1786605663</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786734900</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>197.735862</t>
+          <t>289.839572</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,39 +1179,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
+          <t>0xd64487136d220bcde0c34443c28dae20b7ce8df92715349e80439bb3add91afd</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x960070fC76573ff9c086dB473f99CA99ea914dd6</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.29</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4563</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1203,27 +1211,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Udinese Calcio vs Padova</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Udinese Calcio</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x675ece5a0474a0ced0be4a5ccf3d6cab66f0ec277bf57fac8456b452ec7fd3de</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19758479</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1248,17 +1256,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786301791</t>
+          <t>1786559970</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786811400</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>22.553425</t>
+          <t>9.056604</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,31 +1283,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
+          <t>0xfd452d709e743a453967c2f09f915be8bf7b3736a08df29863146a0def6fb8b9</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.78999</t>
+          <t>98.93</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5613</t>
+          <t>1.5725</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Benevento Calcio -1</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1307,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
+          <t>0xce3150e284359bf496f40ccdc388bb1fabe425bbbbaef33748712f56a7829f8b</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1352,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786296460</t>
+          <t>1786308240</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>22.788401</t>
+          <t>172.803493</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,28 +1395,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
+          <t>0x8aae10e1709c5b66d3944742ea49c3f34481d8efcc4a674cbe430d4c8ecadc0c</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x49c03d69c92f4aEa65FBF1F149A1ac3Bf31A37C6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.64948</t>
+          <t>34.28</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1411,27 +1427,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
+          <t>0xb37240201708d25dc56c7c5e8b0026a7fcf703c38ba73d39f50359efc04be8ba</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1456,17 +1472,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786296207</t>
+          <t>1786303449</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>48.5395</t>
+          <t>62.327273</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1483,28 +1499,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
+          <t>0x8fb36da59c4b6bd10996dd73aefec25b583a3b881c459a65356ac312aaac3fa0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22.73178</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.4338</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1515,27 +1531,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1560,17 +1576,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786296110</t>
+          <t>1786302954</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>11.527378</t>
+          <t>313.541793</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1587,62 +1603,54 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
+          <t>0xea19f3d7c8aed58ad72ca577cca6e8816443dccd75fdbfeb2ccdb152b052b53b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>14.33585</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Arezzo vs Union Brescia</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Arezzo</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>Union Brescia</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Arezzo vs Union Brescia</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Arezzo</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x85827689adea8a2163518b009637621afe8cd3bbdc964b5a5ebf8051f7e81526</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1672,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786295837</t>
+          <t>1786302861</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1682,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>197.735862</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1699,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
+          <t>0x21db31cdab3baa2bdeaed2b17082de81495b504524b4ff74a9fc2180a4398a5d</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1714,22 +1722,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>10.29</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.4563</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Benevento Calcio -1.5</t>
+          <t>Arezzo -1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1739,27 +1747,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1784,17 +1792,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786293531</t>
+          <t>1786301791</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>27.04918</t>
+          <t>22.553425</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1811,39 +1819,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
+          <t>0xc386d94ecfeacaa8164f0f1bb997f6e256828f15da7fd40676bd859fa20a713f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>6.405</t>
+          <t>12.78999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.305</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Benevento Calcio -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1851,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
+          <t>0x0547057ad2972baab22722af2264f8c3e16f62a5975275dfdcb4377b7a1cd5e7</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786293491</t>
+          <t>1786296460</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>22.788401</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,7 +1923,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
+          <t>0x33e275e2954e140f5b351b9f3fd5f66a507ae84b9868de785de6742a058977e4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1931,31 +1931,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>11.64948</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Arezzo -1.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -1963,27 +1955,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0x64dc70073c465071dc1517d9104eb3b826ff9441c071d67535c7c9d3ece7b9ff</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2008,17 +2000,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786296207</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>48.5395</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,39 +2027,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
+          <t>0x616957c3b580994d88ac16565205f196a7ea047493adff86f04b26285a19bf22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.07162</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Arezzo -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2075,27 +2059,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x72ddbc76c1375caa2e0960e666f8f5e795c7c9292e9b70a4856c51d29a1ec7f8</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2120,17 +2104,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786293490</t>
+          <t>1786296110</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>3.987423</t>
+          <t>11.527378</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2147,7 +2131,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
+          <t>0x40180a34b18ad14ba3e1f3e0ce6f495e1ad8a2c236a1fa672db717c4268949b8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2162,22 +2146,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Arezzo -1.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2202,7 +2186,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2232,7 +2216,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786293441</t>
+          <t>1786295837</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2242,7 +2226,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>48.09816</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2259,12 +2243,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
+          <t>0xcfeb7852787d2f7fa9afd6a86dee4ac81c269ff30125bc2a38a43f7369eee202</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E10BB517d5F2D4B81D412613c485Dfa4988F205</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2274,22 +2258,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11.63</t>
+          <t>8.25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Arezzo -1</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2299,27 +2283,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2344,17 +2328,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786293440</t>
+          <t>1786293531</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>43.274419</t>
+          <t>27.04918</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2371,12 +2355,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
+          <t>0xbc8d1328a65f7a31921449e0189a718c1398127895a936c87c01eb552c41c57f</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAAC601FEf8F6FBd4D17d515dA528e648f468E0A1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2386,7 +2370,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>14.66</t>
+          <t>6.405</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2456,7 +2440,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786293437</t>
+          <t>1786293491</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2466,7 +2450,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>48.065574</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2483,7 +2467,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
+          <t>0xa6b3f24dc16debae1e903d172350bc7891153755038d4d356ee84ba06a9b0e0b</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2498,22 +2482,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.53638</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Arezzo -1.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2523,27 +2507,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Benevento Calcio vs Ravenna</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Benevento Calcio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Ravenna</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19721150</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2568,17 +2552,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786293128</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786302000</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>13.536383</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2595,7 +2579,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
+          <t>0xa66022cf08e4a937a81d8886a3e8333c6105b956f6eeeafea8f983dbcd07c7a8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2610,47 +2594,47 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>1.07162</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Arezzo vs Union Brescia</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Arezzo</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>Union Brescia</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Arezzo vs Union Brescia</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Arezzo</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Union Brescia</t>
-        </is>
-      </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2680,7 +2664,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786293055</t>
+          <t>1786293490</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2674,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>12.76</t>
+          <t>3.987423</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,31 +2691,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
+          <t>0xdaa693bb8f1aa61e4c43e39181aea6451ffd67a9357643ba25dd113dad652ca2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Arezzo -1.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2754,7 +2746,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0x97d4833dd740e9c5281dd24875b91a8a9abbc02a6a55eddefe6955b183815e2e</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2784,7 +2776,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786277299</t>
+          <t>1786293441</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2786,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>48.09816</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,31 +2803,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
+          <t>0x904289494cb2be336b1ffbc96c4b7b49556c6e1022088f2e9eb88ab79952e57a</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11.63</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.7563</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Arezzo -1</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
+          <t>0xdac993766cc895cd89576232f9c256563080f60bd9b42bccb3a4714fdae596ae</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786277209</t>
+          <t>1786293440</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>6.61157</t>
+          <t>43.274419</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2915,12 +2915,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
+          <t>0x2a501ac5d083ad687b60d3b46cef3fc6a21f44303ff420b077a53a43b3175c77</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2930,22 +2930,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>31.81</t>
+          <t>14.66</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.6625</t>
+          <t>1.305</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Arezzo 0</t>
+          <t>Benevento Calcio -1.5</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2955,27 +2955,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
+          <t>0x7681bbb2329149b1bd048aad9a7d61e10dbb9076d0a7ff0d3c64244a80a7fb88</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3000,17 +3000,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786262452</t>
+          <t>1786293437</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>48.015094</t>
+          <t>48.065574</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3027,7 +3027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
+          <t>0x49434e79fa99775e1d8fc3cf10b76620b3c40cfc254155950a89ac28cc16f9c9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3042,22 +3042,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>12.50625</t>
+          <t>3.53638</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3067,27 +3067,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Arezzo vs Union Brescia</t>
+          <t>Benevento Calcio vs Ravenna</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Arezzo</t>
+          <t>Benevento Calcio</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Union Brescia</t>
+          <t>Ravenna</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0x941bf8ec1250d230c73720d0b2047b938f4839014b5ffd493767dd9348c728a4</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19721153</t>
+          <t>L19721150</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3112,17 +3112,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786260986</t>
+          <t>1786293128</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786297500</t>
+          <t>1786302000</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>13.536383</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3139,7 +3139,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
+          <t>0x962538877b77d3c65ee91ff655def8edb11073878bf6706f56a062cac9580cd6</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3154,22 +3154,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>7.83</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4312</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786256291</t>
+          <t>1786293055</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>18.156522</t>
+          <t>12.76</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,28 +3251,28 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
+          <t>0x0f5e7aa0a78b72175375b70f9aa8345808f0018dc8930c6d2ef84afea2e4fec1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>16.637</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -3283,27 +3283,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3328,17 +3328,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786277299</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>71.556989</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3355,28 +3355,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
+          <t>0xa269c27d4209de50f5024f7d2b3c5e8025d3dc69d33aee153f9771e38a97380f</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>224.19362</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.7563</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3387,27 +3387,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xa4e26f66e94bd9b427d7db7a5daf9916aea57a1ef7e6ac179358a37c941a1454</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3432,17 +3432,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786219001</t>
+          <t>1786277209</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>964.273634</t>
+          <t>6.61157</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3459,12 +3459,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
+          <t>0xe5d9fc057faaec093ce083d1797731dc8b594ffb03ad681118a742d4a7d06901</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3474,22 +3474,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>14.32754</t>
+          <t>31.81</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.1675</t>
+          <t>1.6625</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Arezzo 0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3499,27 +3499,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0x54c0ae6b2003bf79d6989e9c0e786870ba76f797b5bf795d54dcf7bed7ac726e</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3544,17 +3544,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786218965</t>
+          <t>1786262452</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>85.537552</t>
+          <t>48.015094</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3571,12 +3571,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
+          <t>0x833356fdcb6c8dec55dc5d7df816b5e85e5a28f98cec4582369d2e96e0b49a7e</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3586,22 +3586,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>12.50625</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.2763</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3611,27 +3611,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3656,17 +3656,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786217596</t>
+          <t>1786260986</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>96.39819</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3683,12 +3683,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
+          <t>0x3c91a66b2b62c8154322f9b1dbcd74f7279f54d773764598acfebcd30d43b796</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3698,22 +3698,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>20.79</t>
+          <t>7.83</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.4312</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3723,27 +3723,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Arezzo vs Union Brescia</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Union Brescia</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
+          <t>0xe2a74d4aa3b774c3eb9fa12d33c61153eb53cae5a5dd7cc6ee2a713bda152b88</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721153</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3768,17 +3768,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786217152</t>
+          <t>1786256291</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786297500</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>18.156522</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3795,7 +3795,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
+          <t>0x7b82138cf377d8f66c082c7e9d873d8596ee63c3e8df3b93bf0a6d29736b07eb</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3803,19 +3803,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>175.30999</t>
+          <t>16.637</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3823,11 +3819,7 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Vicenza 0</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3835,27 +3827,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3880,17 +3872,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>266.125222</t>
+          <t>71.556989</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3907,7 +3899,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
+          <t>0x587fd2e1314ee2479847c52a336aab8441d4b0bdc7f6e65809ac68caa2fa10db</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3915,19 +3907,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>261.74</t>
+          <t>224.19362</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3935,11 +3923,7 @@
           <t>Coppa Italia</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Vicenza</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -3947,27 +3931,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3992,17 +3976,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786216909</t>
+          <t>1786219001</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>397.328273</t>
+          <t>964.273634</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4019,7 +4003,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
+          <t>0x551340ab735edb0b9b006fe7400c792652876315e9708a08b5a2dbe930841a3a</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4034,22 +4018,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>15.57</t>
+          <t>14.32754</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.1675</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Ascoli Picchio -1.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4074,7 +4058,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4104,7 +4088,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786216868</t>
+          <t>1786218965</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4114,7 +4098,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>85.315068</t>
+          <t>85.537552</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4131,7 +4115,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
+          <t>0xa7a2b2fd033daab3f00ab3f88c94403dd7c454babf17956ca4b42c291cc15f38</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4146,12 +4130,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>18.08</t>
+          <t>26.63</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.2763</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4216,7 +4200,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786216686</t>
+          <t>1786217596</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4226,7 +4210,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>67.906103</t>
+          <t>96.39819</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4243,31 +4227,39 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
+          <t>0xc7412334a384b68c759daa6a533cf7ccf4975275e54d8e63cb6b2c6b04b8e0f4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>27.61</t>
+          <t>20.79</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.2363</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4290,7 +4282,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4320,7 +4312,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786215506</t>
+          <t>1786217152</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4330,7 +4322,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>116.867725</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4347,12 +4339,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
+          <t>0x9824db72136003c391fed9d3b284dfe343113787d9d57d9b9a9e679b29f47c38</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4362,22 +4354,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>436.64999</t>
+          <t>175.30999</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Vicenza 0</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4402,7 +4394,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
+          <t>0x1e11eb9a8201cb1f1f2c44276645f0ae6a80e30239a2927d9f0aedc687e9cb03</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4432,7 +4424,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786214910</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4442,7 +4434,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>771.12581</t>
+          <t>266.125222</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4459,12 +4451,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
+          <t>0x3b0e49cd69b16eedf311a91a55e251b833ecde2864151d02a107eaf5029a3c28</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4474,12 +4466,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>13.08</t>
+          <t>261.74</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4489,7 +4481,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio 0</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4499,27 +4491,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4544,17 +4536,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786214365</t>
+          <t>1786216909</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>24.166282</t>
+          <t>397.328273</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4571,31 +4563,39 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
+          <t>0xf7f2f2450aee57586d0ccf540e6ad017c2a0cf688186efa84c11f4dd7f7d5137</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.28999</t>
+          <t>15.57</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.7175</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio -1.5</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
+          <t>0x8ed4397196b17ed5bb1e6b153cfecb41f37185dc77142f2887059028a3da449c</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786214242</t>
+          <t>1786216868</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>4.585352</t>
+          <t>85.315068</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4675,12 +4675,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
+          <t>0xa6e375fe5f3477de238d7d3d8f4cdb19357538dc0d9b228c7adf08e2c7c2f67b</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4690,22 +4690,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18.08</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Ascoli Picchio -1</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4715,27 +4715,27 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
+          <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4760,17 +4760,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786211540</t>
+          <t>1786216686</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>21.978022</t>
+          <t>67.906103</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4787,39 +4787,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
+          <t>0xd10abc1712864366f632b091c893868974a708c60c390618d4152ac702edfcbf</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>49.90995</t>
+          <t>27.61</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.7388</t>
+          <t>1.2363</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -4842,7 +4834,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4872,7 +4864,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786211170</t>
+          <t>1786215506</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4882,7 +4874,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>67.56</t>
+          <t>116.867725</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4899,12 +4891,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
+          <t>0xd567a1601c6d1d3131d2cd468fa7f1c3f5b3e63f40c8673dac85e3503491a2a5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4914,22 +4906,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>5.48</t>
+          <t>436.64999</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4954,7 +4946,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x984b3ed1c06f940956d40875fe5c4990316e0067a7ee9f6c01a5d487467bc613</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4984,7 +4976,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786206603</t>
+          <t>1786214910</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4994,7 +4986,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>18.190871</t>
+          <t>771.12581</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5011,12 +5003,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
+          <t>0x9cd7761be82664bdcb28fe5f2b7af687a7b9b707a3ae89dd0cda82b93e8ad8da</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5026,22 +5018,22 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.42844</t>
+          <t>13.08</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Coppa Italia</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Vicenza -1.5</t>
+          <t>Ascoli Picchio 0</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -5051,27 +5043,27 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0xa9259799d9f108a8bde25be876bcff9121f1df206f8effe37102d2103808d83b</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -5096,17 +5088,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786206465</t>
+          <t>1786214365</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1.422207</t>
+          <t>24.166282</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5123,7 +5115,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+          <t>0x722da7f8c22b394edf109669e6ddcbbdd56845facce03f86864efee67f7b68b2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5131,31 +5123,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>3.28999</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.3013</t>
+          <t>1.7175</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Vicenza -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5163,27 +5147,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Vicenza vs Catania</t>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Ascoli Picchio</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Catania</t>
+          <t>Potenza Calcio</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+          <t>0x5c5307ef06cb2727d8a2466836eac51e8c2bd9ff67800f9149bf2000d7b92e79</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>L19721151</t>
+          <t>L19721152</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5208,17 +5192,17 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786206249</t>
+          <t>1786214242</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>1786212000</t>
+          <t>1786213800</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>16.298755</t>
+          <t>4.585352</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,31 +5219,39 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+          <t>0x5ccdf8dbbc91f477d6e580265065ea3d78a2af91c12a37783d5fc54e81618832</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>9.59075</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5267,27 +5259,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+          <t>0xddcebc643cafe51cc5600202a42a67cb8bdcc5ee89b451de170a5dfba49b2560</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5312,17 +5304,17 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786204683</t>
+          <t>1786211540</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>48.560759</t>
+          <t>21.978022</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5339,31 +5331,39 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+          <t>0xcc94d48829914d41645d04b4ac4d025cd51699f39559811921f035daace2591f</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>11.94608</t>
+          <t>49.90995</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.7388</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0xc8bddb4152e6149344fbfa8473b10a9ef4134ba63c821197df363d18a89b2f21</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1786204434</t>
+          <t>1786211170</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>13.99248</t>
+          <t>67.56</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5443,7 +5443,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+          <t>0x287cb6a6fee69cee3d7fe218a74dd703ce9cab8814d7e817726d852f8f9520dc</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5451,23 +5451,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>46.42999</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.8538</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5475,27 +5483,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Ascoli Picchio vs Potenza Calcio</t>
+          <t>Vicenza vs Catania</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Ascoli Picchio</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Potenza Calcio</t>
+          <t>Catania</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>L19721152</t>
+          <t>L19721151</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5520,17 +5528,17 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1786204373</t>
+          <t>1786206603</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>1786213800</t>
+          <t>1786212000</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>54.38359</t>
+          <t>18.190871</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5547,31 +5555,39 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+          <t>0x7ebdb840ed671a775e550cae8c5617ee0efa4676795d6acdc2956fcf4135845c</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>15.84</t>
+          <t>0.42844</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.3013</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>Coppa Italia</t>
@@ -5594,7 +5610,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5624,7 +5640,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1786194158</t>
+          <t>1786206465</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5634,7 +5650,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>64.984615</t>
+          <t>1.422207</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5651,110 +5667,638 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>0xa95818308c965c64dd4d898039674feded4b06aca9c48b3bbc7c0f14dab56b21</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>4.91</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.3013</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Vicenza -1.5</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x4d7b719c019ec7e29612fd8e5ba567502af8e6c9d3f680a333a9c38c1d213170</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1786206249</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>16.298755</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0xf84f003a4c78b0e9a6719c288a729c4aa1384b3c69a07a817a5faec75ec5f915</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>9.59075</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.1975</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0xc5cf82c8a5697ef431004a29f0d5f57c29a47c794d91db5ed3fe77634082651d</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1786204683</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>48.560759</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0x5b2bb58020d7f81ee65e784fb8aa9c87b68178ab630cbde0aa88bc4982e6770a</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>11.94608</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1786204434</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>13.99248</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0x81b3829aecfb0da93f104b75018585829e653eb863a413b881c63cc605880a57</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>46.42999</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1.8538</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio vs Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Ascoli Picchio</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Potenza Calcio</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>0x0ce62fd21140857b7b0f61adcffd727d3d134f980f49abc34f90c69a7b5ea6e3</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>L19721152</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>1786204373</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>1786213800</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>54.38359</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0xe6f24003437483927b7465d8497187c5f3e54d727b812eed867c346cc248c844</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>15.84</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1.2437</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Vicenza vs Catania</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Vicenza</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Catania</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>0x6053c51246e76b7ad939ccdca60bb74113673c3eb2bde5c5d148430ae5f65338</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>L19721151</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>1786194158</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>1786212000</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>64.984615</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>0x3a760c290056c65523a32099d57699c45f7ef42b14c3cb07eb55dbfffa62aaef</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>12.85165</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>1.5038</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>Ascoli Picchio -1</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Coppa Italia</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Coppa Italia</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
         <is>
           <t>Ascoli Picchio vs Potenza Calcio</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>Ascoli Picchio</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>Potenza Calcio</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>0xd05207b576f199de4cabc6f042bd126d107c8d4c10008a2809194a2d93f44b7c</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>L19721152</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
         <is>
           <t>1786165402</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="S54" t="inlineStr">
         <is>
           <t>1786213800</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>25.51196</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr">
+      <c r="V54" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>